<commit_message>
chore: dae_il 및 Braintree 감사 자동화 전체 실행 결과물 업데이트 (20260511)
- dae_il: run.js → data_injector → interest_expense_extractor → interest_expense_analysis 순차 실행 완료
- dae_il/results: 20260511 날짜 결과 파일 신규 생성
- dae_il/results: 이자비용적정성.xlsx, 이자비용분석결과.xlsx 생성
- dae_il 감사조서 updated.xlsx 업데이트
- Braintree: raw_data 파일명 변경 (당기/전기 구분), 20260421 결과 삭제 → 20260504 결과 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Braintree/task_list_braintree.xlsx
+++ b/Braintree/task_list_braintree.xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\lbh00\OneDrive\문서\감사\감사자료\audit-automation\Braintree\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9601E2-14D5-4E8B-B277-A906E1E942F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AABC61B-657B-49A8-9530-2803087AA308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="12196" activeTab="3" xr2:uid="{0988228D-CB65-49FF-A818-8D2DE82566F6}"/>
+    <workbookView xWindow="-19298" yWindow="-98" windowWidth="19396" windowHeight="12196" firstSheet="3" activeTab="4" xr2:uid="{0988228D-CB65-49FF-A818-8D2DE82566F6}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
     <sheet name="host1_총계정원장" sheetId="2" r:id="rId2"/>
     <sheet name="host1_상세검색_시나리오" sheetId="3" r:id="rId3"/>
     <sheet name="host1_벤포드법칙분석" sheetId="5" r:id="rId4"/>
-    <sheet name="host2_분개장AI분석" sheetId="4" r:id="rId5"/>
+    <sheet name="host1_전기 데이터 비교 분석" sheetId="8" r:id="rId5"/>
+    <sheet name="host1_이중거래처분석" sheetId="6" r:id="rId6"/>
+    <sheet name="host1_외상매출매입상계" sheetId="7" r:id="rId7"/>
+    <sheet name="host2_분개장AI분석" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="52">
   <si>
     <t>항목</t>
   </si>
@@ -230,6 +233,10 @@
   </si>
   <si>
     <t>분석할 계정과목</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>지급수수료</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1024,6 +1031,65 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{265A6539-2564-46BF-942B-EEC385B53B6D}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.08203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D14481-7FF3-4693-99E5-2CB88F450E06}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F26966BA-9AA6-46A4-A0FC-D608B070C3C3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E4E540D-2F54-444B-8CC0-15566B81F298}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>

</xml_diff>